<commit_message>
chore: update stufe-5/med/extract-amts-from-ig-ptdata-1884 pages
</commit_message>
<xml_diff>
--- a/stufe-5/med/extract-amts-from-ig-ptdata-1884/ValueSet-current-smoking-status-uv-ips.xlsx
+++ b/stufe-5/med/extract-amts-from-ig-ptdata-1884/ValueSet-current-smoking-status-uv-ips.xlsx
@@ -36,7 +36,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.0.1</t>
+    <t>6.0.0-rc</t>
   </si>
   <si>
     <t>Name</t>
@@ -66,7 +66,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-08T14:03:32+00:00</t>
+    <t>2026-01-08T14:46:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>